<commit_message>
feat(storage): dual backend with postgres persistence for production and excel for local dev
</commit_message>
<xml_diff>
--- a/data/jobs.backup.xlsx
+++ b/data/jobs.backup.xlsx
@@ -1369,17 +1369,17 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
     </row>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-28 23:21:42</t>
+          <t>2026-10-29 13:26:25</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-10-28 23:21:42</t>
+          <t>2026-10-29 13:26:25</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -2161,7 +2161,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-10-28 23:21:43</t>
+          <t>2026-10-29 13:26:26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">

</xml_diff>